<commit_message>
docs: N14 setPending 입력 필드 이름 확정, 명세 v16 (#33)
* docs: N14 setPending 입력 필드 이름 확정, 명세 v16

* docs: 명세 v16 파일을 서식·계산 값 그대로 다시 저장
</commit_message>
<xml_diff>
--- a/docs/spec.xlsx
+++ b/docs/spec.xlsx
@@ -53,7 +53,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2026-10-25 · v15 (v2: </t>
+      <t xml:space="preserve">2026-10-29 · v16 (v2: </t>
     </r>
     <r>
       <rPr>
@@ -1141,7 +1141,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(N24, F10-07) / v15: hasFavicon의 출력을 true·false에서 쓸 파비콘 주소 또는 null로 바꿈. 첫 페이지 주소에서 찾았을 때 appIcon이 그 주소로 그리게 함(N07, N44))</t>
+      <t xml:space="preserve">(N24, F10-07) / v15: hasFavicon의 출력을 true·false에서 쓸 파비콘 주소 또는 null로 바꿈. 첫 페이지 주소에서 찾았을 때 appIcon이 그 주소로 그리게 함(N07, N44) / v16: N14 setPending 입력 필드 이름을 { id, toParentId }로 확정)</t>
     </r>
   </si>
   <si>
@@ -16808,7 +16808,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[{</t>
+      <t xml:space="preserve">[{ id: </t>
     </r>
     <r>
       <rPr>
@@ -16825,6 +16825,40 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">ID, toParentId: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목적지 폴더</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ID }] / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">북마크 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">ID, </t>
     </r>
     <r>
@@ -16833,40 +16867,6 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">목적지 폴더</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">}] / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">북마크 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ID, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">옮겨진 폴더</t>
     </r>
   </si>
@@ -17022,7 +17022,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">옮기기 시작</t>
+      <t xml:space="preserve">옮기기 시작. ID는 문자열로 맞춤. 항목에 id나 toParentId가 없으면 오류.</t>
     </r>
   </si>
   <si>

</xml_diff>